<commit_message>
new test with other percentiles
</commit_message>
<xml_diff>
--- a/test_resultat.xlsx
+++ b/test_resultat.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Desktop\DTU\fagprojekt\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\Desktop\DTU\fagprojekt\Ny mappe\insect-ct-reorientation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{347ED2B1-0AF0-4C5A-A750-CA3B452BE79C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4334D6-6FAB-46A0-823A-D6122B8F8383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{18088B8F-5678-4FBD-8A34-D38BA77D777A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{18088B8F-5678-4FBD-8A34-D38BA77D777A}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -167,13 +167,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" textRotation="45"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -509,9 +508,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045163D2-5EFB-493A-B515-066631FC1948}">
   <dimension ref="A1:P13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:16" ht="79.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="73.2" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
@@ -558,7 +557,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -608,47 +607,47 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3">
         <v>9</v>
       </c>
-      <c r="C3" s="3">
-        <v>10</v>
-      </c>
-      <c r="D3" s="3">
-        <v>10</v>
-      </c>
-      <c r="E3" s="3">
-        <v>10</v>
-      </c>
-      <c r="F3" s="3">
-        <v>10</v>
-      </c>
-      <c r="G3" s="3">
-        <v>10</v>
-      </c>
-      <c r="H3" s="3">
-        <v>10</v>
-      </c>
-      <c r="I3" s="3">
-        <v>10</v>
-      </c>
-      <c r="J3" s="3">
+      <c r="C3">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+      <c r="H3">
+        <v>10</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3">
         <v>7</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3">
         <v>6</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3">
         <v>8</v>
       </c>
-      <c r="M3" s="3">
-        <v>10</v>
-      </c>
-      <c r="N3" s="3">
+      <c r="M3">
+        <v>10</v>
+      </c>
+      <c r="N3">
         <v>10</v>
       </c>
       <c r="O3" s="2"/>
@@ -656,7 +655,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -706,7 +705,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -756,7 +755,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -806,103 +805,103 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7">
         <v>8</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>8</v>
       </c>
-      <c r="D7" s="3">
-        <v>10</v>
-      </c>
-      <c r="E7" s="3">
-        <v>10</v>
-      </c>
-      <c r="F7" s="3">
-        <v>10</v>
-      </c>
-      <c r="G7" s="3">
-        <v>10</v>
-      </c>
-      <c r="H7" s="3">
-        <v>10</v>
-      </c>
-      <c r="I7" s="3">
+      <c r="D7">
+        <v>10</v>
+      </c>
+      <c r="E7">
+        <v>10</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+      <c r="G7">
+        <v>10</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
         <v>8</v>
       </c>
-      <c r="J7" s="3">
+      <c r="J7">
         <v>7</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7">
         <v>6</v>
       </c>
-      <c r="L7" s="3">
-        <v>3</v>
-      </c>
-      <c r="M7" s="3">
-        <v>10</v>
-      </c>
-      <c r="N7" s="3">
+      <c r="L7">
+        <v>3</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+      <c r="N7">
         <v>10</v>
       </c>
       <c r="O7" s="2"/>
-      <c r="P7" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8">
         <v>8</v>
       </c>
-      <c r="C8" s="3">
-        <v>5</v>
-      </c>
-      <c r="D8" s="3">
-        <v>10</v>
-      </c>
-      <c r="E8" s="3">
-        <v>10</v>
-      </c>
-      <c r="F8" s="3">
-        <v>10</v>
-      </c>
-      <c r="G8" s="3">
-        <v>10</v>
-      </c>
-      <c r="H8" s="3">
-        <v>10</v>
-      </c>
-      <c r="I8" s="3">
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8">
+        <v>10</v>
+      </c>
+      <c r="E8">
+        <v>10</v>
+      </c>
+      <c r="F8">
+        <v>10</v>
+      </c>
+      <c r="G8">
+        <v>10</v>
+      </c>
+      <c r="H8">
+        <v>10</v>
+      </c>
+      <c r="I8">
         <v>9</v>
       </c>
-      <c r="J8" s="3">
+      <c r="J8">
         <v>4</v>
       </c>
-      <c r="K8" s="3">
+      <c r="K8">
         <v>6</v>
       </c>
-      <c r="L8" s="3">
+      <c r="L8">
         <v>9</v>
       </c>
-      <c r="M8" s="3">
-        <v>10</v>
-      </c>
-      <c r="N8" s="3">
+      <c r="M8">
+        <v>10</v>
+      </c>
+      <c r="N8">
         <v>10</v>
       </c>
       <c r="O8" s="2"/>
-      <c r="P8" s="3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P8">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -952,7 +951,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1002,27 +1001,55 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
+      <c r="B11" s="2">
+        <v>3</v>
+      </c>
+      <c r="C11" s="2">
+        <v>3</v>
+      </c>
+      <c r="D11" s="2">
+        <v>3</v>
+      </c>
+      <c r="E11" s="2">
+        <v>3</v>
+      </c>
+      <c r="F11" s="2">
+        <v>3</v>
+      </c>
+      <c r="G11" s="2">
+        <v>3</v>
+      </c>
+      <c r="H11" s="2">
+        <v>3</v>
+      </c>
+      <c r="I11" s="2">
+        <v>2</v>
+      </c>
+      <c r="J11" s="2">
+        <v>3</v>
+      </c>
+      <c r="K11" s="2">
+        <v>3</v>
+      </c>
+      <c r="L11" s="2">
+        <v>3</v>
+      </c>
+      <c r="M11" s="2">
+        <v>3</v>
+      </c>
+      <c r="N11" s="2">
+        <v>3</v>
+      </c>
       <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P11" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1072,7 +1099,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Counted results in excel file
</commit_message>
<xml_diff>
--- a/test_resultat.xlsx
+++ b/test_resultat.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bruger\Desktop\DTU\fagprojekt\Ny mappe\insect-ct-reorientation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4334D6-6FAB-46A0-823A-D6122B8F8383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64113E67-ED00-478F-B81C-A2B5678F3CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{18088B8F-5678-4FBD-8A34-D38BA77D777A}"/>
+    <workbookView xWindow="1440" yWindow="1140" windowWidth="21600" windowHeight="11100" xr2:uid="{18088B8F-5678-4FBD-8A34-D38BA77D777A}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>AC</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>Four angles correct</t>
+  </si>
+  <si>
+    <t>PCA</t>
   </si>
 </sst>
 </file>
@@ -507,10 +510,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{045163D2-5EFB-493A-B515-066631FC1948}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:Q14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:16" ht="73.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" ht="73.2" x14ac:dyDescent="0.3">
       <c r="B1" s="1" t="s">
         <v>12</v>
       </c>
@@ -556,8 +559,11 @@
       <c r="P1" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -606,8 +612,11 @@
       <c r="P2">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -654,8 +663,11 @@
       <c r="P3">
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -704,8 +716,11 @@
       <c r="P4">
         <v>10</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -754,8 +769,11 @@
       <c r="P5">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -804,8 +822,11 @@
       <c r="P6">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q6">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -852,8 +873,11 @@
       <c r="P7">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -900,8 +924,11 @@
       <c r="P8">
         <v>10</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -950,8 +977,11 @@
       <c r="P9">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q9">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1000,8 +1030,11 @@
       <c r="P10">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1048,8 +1081,11 @@
       <c r="P11" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q11" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1098,8 +1134,11 @@
       <c r="P12">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="Q12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1147,6 +1186,15 @@
       </c>
       <c r="P13">
         <v>3</v>
+      </c>
+      <c r="Q13">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="Q14">
+        <f>SUM(Q2:Q13)</f>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>